<commit_message>
Update rsvp submissions and simplify app component
Replit-Commit-Author: Agent
</commit_message>
<xml_diff>
--- a/artifacts/api-server/rsvp-submissions.xlsx
+++ b/artifacts/api-server/rsvp-submissions.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="38">
   <si>
     <t>ID</t>
   </si>
@@ -86,6 +86,47 @@
   </si>
   <si>
     <t>Taking photos</t>
+  </si>
+  <si>
+    <t>2026-09-20T09:52:02.376Z</t>
+  </si>
+  <si>
+    <t>Jj</t>
+  </si>
+  <si>
+    <t>0765009671</t>
+  </si>
+  <si>
+    <t>test@gmail.com</t>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yeah
+Noo</t>
+  </si>
+  <si>
+    <t>Groom</t>
+  </si>
+  <si>
+    <t>Eating cake</t>
+  </si>
+  <si>
+    <t>Lol</t>
+  </si>
+  <si>
+    <t>2026-09-21T05:45:00.601Z</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fdfbdfb fd
+fdbfgbfgb</t>
+  </si>
+  <si>
+    <t>All of the above</t>
+  </si>
+  <si>
+    <t>vfdbfdbngf</t>
   </si>
 </sst>
 </file>
@@ -477,7 +518,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L3"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -608,6 +649,82 @@
         <v>14</v>
       </c>
     </row>
+    <row r="4" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2">
+        <v>1789897922376</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="J4" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="L4" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="5" spans="1:12" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="2">
+        <v>1789969500601</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="G5" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="I5" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="J5" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="L5" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:L1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>